<commit_message>
Excel: strip AI-tell glyphs (em/en-dash, middot, times, arrow, approx) to plain ASCII, rename sheet tabs to plain names, update cross-sheet refs + deck sheet-name mention
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Slide15_Investment_Risk_Delivery_Model.xlsx
+++ b/Slide15_Investment_Risk_Delivery_Model.xlsx
@@ -6,18 +6,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="5" activeTab="10" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1 · Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2 · Investment" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3 · Timeline" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4 · Requirements" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5 · Risk register" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6 · ROI" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="12 · Alternatives" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Alt 1 — Own ASIC" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Alt 2 — FPGA" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Alt 3 — ConnectX NIC" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Alt 4 — BlueField-3 (chosen)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="PoC — detail" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="1. Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2. Investment" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="3. Timeline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4. Requirements" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="5. Risk register" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="6. ROI" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="12. Alternatives" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Alt 1 - Own ASIC" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Alt 2 - FPGA" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Alt 3 - ConnectX NIC" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Alt 4 - BlueField-3 (chosen)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="PoC detail" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1151,7 +1151,7 @@
     <row r="1" ht="30" customHeight="1" s="79">
       <c r="A1" s="71" t="inlineStr">
         <is>
-          <t>Quantum Force 9000 — DPU Acceleration Card</t>
+          <t>Quantum Force 9000 - DPU Acceleration Card</t>
         </is>
       </c>
       <c r="B1" s="72" t="n"/>
@@ -1161,10 +1161,11 @@
     <row r="2" ht="17.1" customHeight="1" s="79">
       <c r="A2" s="78" t="inlineStr">
         <is>
-          <t>What it takes to deliver the solution · dynamic investment, risk &amp; delivery model (expanded from Slide 15)</t>
-        </is>
-      </c>
-    </row>
+          <t>What it takes to deliver the solution - dynamic investment, risk &amp; delivery model (expanded from Slide 15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="27.95" customHeight="1" s="79">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -1195,7 +1196,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>TP+TLS: 10.1G → 25G+</t>
+          <t>TP+TLS: 10.1G -&gt; 25G+</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1227,7 +1228,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Not an own ASIC and not a self-designed FPGA — fastest, lowest-risk path</t>
+          <t>Not an own ASIC and not a self-designed FPGA - fastest, lowest-risk path</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1240,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>≈ 4× (10 → ~40G)</t>
+          <t>~ 4x (10 -&gt; ~40G)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1260,7 +1261,7 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>'2 · Investment'!B16</f>
+        <f>'2. Investment'!B16</f>
         <v/>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -1270,7 +1271,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Default rate; individual roles can differ (Investment · drill-down B)</t>
+          <t>Default rate; individual roles can differ (Investment - drill-down B)</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1282,7 @@
         </is>
       </c>
       <c r="B9" s="9">
-        <f>'2 · Investment'!B9</f>
+        <f>'2. Investment'!B9</f>
         <v/>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -1291,7 +1292,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Live link to the Investment total — changes with the inputs</t>
+          <t>Live link to the Investment total - changes with the inputs</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1303,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>'2 · Investment'!B17</f>
+        <f>'2. Investment'!B17</f>
         <v/>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -1323,7 +1324,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>'2 · Investment'!B18</f>
+        <f>'2. Investment'!B18</f>
         <v/>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -1359,6 +1360,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="20.1" customHeight="1" s="79">
       <c r="A14" s="81" t="inlineStr">
         <is>
@@ -1394,15 +1396,15 @@
     <row r="16" ht="15" customHeight="1" s="79">
       <c r="A16" s="86" t="inlineStr">
         <is>
-          <t>R&amp;D · engineers × duration</t>
+          <t>R&amp;D - engineers x duration</t>
         </is>
       </c>
       <c r="B16" s="13">
-        <f>'2 · Investment'!B5</f>
+        <f>'2. Investment'!B5</f>
         <v/>
       </c>
       <c r="C16" s="14">
-        <f>'2 · Investment'!C5</f>
+        <f>'2. Investment'!C5</f>
         <v/>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -1414,15 +1416,15 @@
     <row r="17" ht="15" customHeight="1" s="79">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>HW engineering · thermal · FIPS</t>
+          <t>HW engineering - thermal - FIPS</t>
         </is>
       </c>
       <c r="B17" s="13">
-        <f>'2 · Investment'!B6</f>
+        <f>'2. Investment'!B6</f>
         <v/>
       </c>
       <c r="C17" s="14">
-        <f>'2 · Investment'!C6</f>
+        <f>'2. Investment'!C6</f>
         <v/>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1434,15 +1436,15 @@
     <row r="18" ht="15" customHeight="1" s="79">
       <c r="A18" s="83" t="inlineStr">
         <is>
-          <t>Dev kits · NVIDIA NRE</t>
+          <t>Dev kits - NVIDIA NRE</t>
         </is>
       </c>
       <c r="B18" s="13">
-        <f>'2 · Investment'!B7</f>
+        <f>'2. Investment'!B7</f>
         <v/>
       </c>
       <c r="C18" s="14">
-        <f>'2 · Investment'!C7</f>
+        <f>'2. Investment'!C7</f>
         <v/>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1454,15 +1456,15 @@
     <row r="19" ht="15" customHeight="1" s="79">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>GTM · launch</t>
+          <t>GTM - launch</t>
         </is>
       </c>
       <c r="B19" s="13">
-        <f>'2 · Investment'!B8</f>
+        <f>'2. Investment'!B8</f>
         <v/>
       </c>
       <c r="C19" s="14">
-        <f>'2 · Investment'!C8</f>
+        <f>'2. Investment'!C8</f>
         <v/>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -1478,19 +1480,20 @@
         </is>
       </c>
       <c r="B20" s="13">
-        <f>'2 · Investment'!B9</f>
+        <f>'2. Investment'!B9</f>
         <v/>
       </c>
       <c r="C20" s="14">
-        <f>'2 · Investment'!C9</f>
+        <f>'2. Investment'!C9</f>
         <v/>
       </c>
       <c r="D20" s="13" t="n"/>
     </row>
+    <row r="21"/>
     <row r="22" ht="21.95" customHeight="1" s="79">
       <c r="A22" s="77" t="inlineStr">
         <is>
-          <t>Throughput logic — which numbers are datasheet vs. estimate</t>
+          <t>Throughput logic - which numbers are datasheet vs. estimate</t>
         </is>
       </c>
       <c r="B22" s="74" t="n"/>
@@ -1500,7 +1503,7 @@
     <row r="23" ht="26.1" customHeight="1" s="79">
       <c r="A23" s="73" t="inlineStr">
         <is>
-          <t>9800 published (CP Appliance Chart 2026): 400G raw · 67.7G NGFW · 25G TP · 10.1G TP+TLS.  Only the final ~40G is an estimate — everything else is a datasheet number, and the multiples are just division.</t>
+          <t>9800 published (CP Appliance Chart 2026): 400G raw - 67.7G NGFW - 25G TP - 10.1G TP+TLS. Only the final ~40G is an estimate - everything else is a datasheet number, and the multiples are just division.</t>
         </is>
       </c>
       <c r="B23" s="74" t="n"/>
@@ -1532,7 +1535,7 @@
     <row r="25" ht="26.1" customHeight="1" s="79">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Today — on the x86</t>
+          <t>Today - on the x86</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
@@ -1559,7 +1562,7 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>25G → 10.1G</t>
+          <t>25G -&gt; 10.1G</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
@@ -1576,7 +1579,7 @@
     <row r="27" ht="26.1" customHeight="1" s="79">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Offload TLS → BF-3</t>
+          <t>Offload TLS -&gt; BF-3</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
@@ -1598,7 +1601,7 @@
     <row r="28" ht="26.1" customHeight="1" s="79">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Offload IPS (RXP) → BF-3</t>
+          <t>Offload IPS (RXP) -&gt; BF-3</t>
         </is>
       </c>
       <c r="B28" s="20" t="inlineStr">
@@ -1625,7 +1628,7 @@
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>≈ 4×</t>
+          <t>~ 4x</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
@@ -1647,7 +1650,7 @@
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>25G+ (2.5×)</t>
+          <t>25G+ (2.5x)</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
@@ -1664,7 +1667,7 @@
     <row r="31" ht="39.95" customHeight="1" s="79">
       <c r="A31" s="76" t="inlineStr">
         <is>
-          <t>Bottom line: 10.1G and 25G are the 9800’s own datasheet numbers; offloading TLS just returns you to 25G. Offloading IPS is the estimated step that adds the rest to ~40G — bounded above by the 67.7G NGFW figure and limited by x86 policy. The PoC validates that single soft number.</t>
+          <t>Bottom line: 10.1G and 25G are the 9800's own datasheet numbers; offloading TLS just returns you to 25G. Offloading IPS is the estimated step that adds the rest to ~40G - bounded above by the 67.7G NGFW figure and limited by x86 policy. The PoC validates that single soft number.</t>
         </is>
       </c>
       <c r="B31" s="74" t="n"/>
@@ -1675,7 +1678,7 @@
     <row r="33" ht="21.95" customHeight="1" s="79">
       <c r="A33" s="80" t="inlineStr">
         <is>
-          <t>Check Point Software Technologies · Confidential   |   Barak Rozenfeld · Senior PM Assignment 2026   |   Slide 15   |   Cream = editable input · grey = formula (recalculates).</t>
+          <t>Check Point Software Technologies - Confidential | Barak Rozenfeld - Senior PM Assignment 2026 | Slide 15 | Cream = editable input - grey = formula (recalculates).</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1723,7 @@
     <row r="1" ht="16.5" customHeight="1" s="79">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>Alternative 3 — Use a ConnectX-7 SmartNIC</t>
+          <t>Alternative 3 - Use a ConnectX-7 SmartNIC</t>
         </is>
       </c>
     </row>
@@ -1731,6 +1734,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="55" t="inlineStr">
         <is>
@@ -1802,7 +1806,7 @@
       </c>
       <c r="B8" s="59" t="inlineStr">
         <is>
-          <t>10 → ~20 (×2)</t>
+          <t>10 -&gt; ~20 (x2)</t>
         </is>
       </c>
       <c r="C8" s="96" t="inlineStr">
@@ -1828,6 +1832,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="55" t="inlineStr">
         <is>
@@ -1908,6 +1913,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="55" t="inlineStr">
         <is>
@@ -1940,7 +1946,7 @@
     <row r="19">
       <c r="A19" s="61" t="inlineStr">
         <is>
-          <t>FTE — integration team</t>
+          <t>FTE - integration team</t>
         </is>
       </c>
       <c r="B19" s="70" t="n">
@@ -2035,7 +2041,7 @@
       </c>
       <c r="C25" s="95" t="inlineStr">
         <is>
-          <t>Lighter — reusing a shipping NIC</t>
+          <t>Lighter - reusing a shipping NIC</t>
         </is>
       </c>
     </row>
@@ -2112,17 +2118,18 @@
     <row r="1" ht="16.5" customHeight="1" s="79">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>Alternative 4 — Use a BlueField-3 acceleration card  ✓ CHOSEN</t>
+          <t>Alternative 4 - Use a BlueField-3 acceleration card ✓ CHOSEN</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" s="79">
       <c r="A2" s="94" t="inlineStr">
         <is>
-          <t>An existing NVIDIA BlueField-3 card in a Check Point-format slot. Chosen: best throughput per RU without sacrificing flexibility — a new engine (incl. AI/ML) ships as a software update, and BF-3 is already proven in Check Point AI Cloud Protect (AIFF). Cream = editable input · grey = formula.</t>
-        </is>
-      </c>
-    </row>
+          <t>An existing NVIDIA BlueField-3 card in a Check Point-format slot. Chosen: best throughput per RU without sacrificing flexibility - a new engine (incl. AI/ML) ships as a software update, and BF-3 is already proven in Check Point AI Cloud Protect (AIFF). Cream = editable input - grey = formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="55" t="inlineStr">
         <is>
@@ -2194,12 +2201,12 @@
       </c>
       <c r="B8" s="62" t="inlineStr">
         <is>
-          <t>10 → ~40 (×4)</t>
+          <t>10 -&gt; ~40 (x4)</t>
         </is>
       </c>
       <c r="C8" s="96" t="inlineStr">
         <is>
-          <t>Offloads TLS crypto + IPS; PoC gate is a conservative 25G+ (×2.5)</t>
+          <t>Offloads TLS crypto + IPS; PoC gate is a conservative 25G+ (x2.5)</t>
         </is>
       </c>
     </row>
@@ -2220,6 +2227,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="55" t="inlineStr">
         <is>
@@ -2296,10 +2304,11 @@
       </c>
       <c r="C15" s="95" t="inlineStr">
         <is>
-          <t>Not from scratch — the 9000 already runs acceleration cards; BF-3 is in AIFF</t>
-        </is>
-      </c>
-    </row>
+          <t>Not from scratch - the 9000 already runs acceleration cards; BF-3 is in AIFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="55" t="inlineStr">
         <is>
@@ -2370,7 +2379,7 @@
       </c>
       <c r="C21" s="95" t="inlineStr">
         <is>
-          <t>≈ $250K / engineer-year, fully loaded</t>
+          <t>~ $250K / engineer-year, fully loaded</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2467,7 @@
       </c>
       <c r="C27" s="95" t="inlineStr">
         <is>
-          <t>Sums to ~$7.0M. The full program on '2 · Investment' is $7.2M (adds HW/FIPS + GTM beyond this R&amp;D+PoC core)</t>
+          <t>Sums to ~$7.0M. The full program on '2 - Investment' is $7.2M (adds HW/FIPS + GTM beyond this R&amp;D+PoC core)</t>
         </is>
       </c>
     </row>
@@ -2505,17 +2514,18 @@
     <row r="1">
       <c r="A1" s="109" t="inlineStr">
         <is>
-          <t>PoC — detailed plan (investment structure + effort timeline)</t>
+          <t>PoC - detailed plan (investment structure + effort timeline)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" s="79">
       <c r="A2" s="110" t="inlineStr">
         <is>
-          <t>The $2.9M / ~6-month Proof-of-Concept that must clear ONE gate (25 Gbps+ under TLS) before the $4.3M GA spend is released.  Cream = editable input · grey = formula (recalculates).</t>
-        </is>
-      </c>
-    </row>
+          <t>The $2.9M / ~6-month Proof-of-Concept that must clear ONE gate (25 Gbps+ under TLS) before the $4.3M GA spend is released. Cream = editable input - grey = formula (recalculates).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="97" t="inlineStr">
         <is>
@@ -2552,7 +2562,7 @@
       </c>
       <c r="B6" s="111" t="inlineStr">
         <is>
-          <t>25 Gbps+ under TLS (×2.5)</t>
+          <t>25 Gbps+ under TLS (x2.5)</t>
         </is>
       </c>
       <c r="C6" s="112" t="inlineStr">
@@ -2624,14 +2634,15 @@
       </c>
       <c r="C10" s="112" t="inlineStr">
         <is>
-          <t>Released only if the gate is met — otherwise we stop</t>
-        </is>
-      </c>
-    </row>
+          <t>Released only if the gate is met - otherwise we stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="97" t="inlineStr">
         <is>
-          <t>Investment structure · PoC — bottom-up to $2.9M</t>
+          <t>Investment structure - PoC - bottom-up to $2.9M</t>
         </is>
       </c>
       <c r="B12" s="98" t="n"/>
@@ -2657,7 +2668,7 @@
       </c>
       <c r="E14" s="106" t="inlineStr">
         <is>
-          <t>Focused subset — core offload + driver + perf</t>
+          <t>Focused subset - core offload + driver + perf</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2709,7 @@
     <row r="17">
       <c r="A17" s="104" t="inlineStr">
         <is>
-          <t>R&amp;D subtotal  =  engineers × months × rate</t>
+          <t>R&amp;D subtotal = engineers x months x rate</t>
         </is>
       </c>
       <c r="D17" s="102">
@@ -2707,10 +2718,11 @@
       </c>
       <c r="E17" s="106" t="inlineStr">
         <is>
-          <t>≈ $1.25M</t>
-        </is>
-      </c>
-    </row>
+          <t>~ $1.25M</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="100" t="inlineStr">
         <is>
@@ -2955,7 +2967,7 @@
     <row r="30">
       <c r="A30" s="104" t="inlineStr">
         <is>
-          <t>TOTAL PoC  =  R&amp;D + non-R&amp;D</t>
+          <t>TOTAL PoC = R&amp;D + non-R&amp;D</t>
         </is>
       </c>
       <c r="D30" s="113">
@@ -2964,14 +2976,15 @@
       </c>
       <c r="E30" s="106" t="inlineStr">
         <is>
-          <t>≈ $2.9M  (phase-slice of the $7.2M full program)</t>
-        </is>
-      </c>
-    </row>
+          <t>~ $2.9M (phase-slice of the $7.2M full program)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="97" t="inlineStr">
         <is>
-          <t>Effort timeline · PoC — phases sum to ~6 months</t>
+          <t>Effort timeline - PoC - phases sum to ~6 months</t>
         </is>
       </c>
       <c r="B32" s="98" t="n"/>
@@ -3009,7 +3022,7 @@
       </c>
       <c r="D34" s="99" t="inlineStr">
         <is>
-          <t>Set up BF-3 boards, lab and baseline — environment ready</t>
+          <t>Set up BF-3 boards, lab and baseline - environment ready</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3037,7 @@
       </c>
       <c r="D35" s="99" t="inlineStr">
         <is>
-          <t>DOCA/Gaia driver + CoreXL offload path — TLS path running on the card</t>
+          <t>DOCA/Gaia driver + CoreXL offload path - TLS path running on the card</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3052,7 @@
       </c>
       <c r="D36" s="99" t="inlineStr">
         <is>
-          <t>Measure TP under TLS and tune — the make-or-break gate</t>
+          <t>Measure TP under TLS and tune - the make-or-break gate</t>
         </is>
       </c>
     </row>
@@ -3054,7 +3067,7 @@
       </c>
       <c r="D37" s="99" t="inlineStr">
         <is>
-          <t>1RU thermal sim + FIPS path — headroom &amp; cert path confirmed</t>
+          <t>1RU thermal sim + FIPS path - headroom &amp; cert path confirmed</t>
         </is>
       </c>
     </row>
@@ -3070,10 +3083,11 @@
       </c>
       <c r="D38" s="106" t="inlineStr">
         <is>
-          <t>≈ 6 months to the gate</t>
-        </is>
-      </c>
-    </row>
+          <t>~ 6 months to the gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="97" t="inlineStr">
         <is>
@@ -3093,7 +3107,7 @@
       </c>
       <c r="B41" s="112" t="inlineStr">
         <is>
-          <t>≥ 25 Gbps TP under TLS (×2.5 vs 10G today) — the go/no-go number</t>
+          <t>&gt;= 25 Gbps TP under TLS (x2.5 vs 10G today) - the go/no-go number</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3143,7 @@
       </c>
       <c r="B44" s="112" t="inlineStr">
         <is>
-          <t>FIPS 140-3 path confirmed — BF-3 crypto module already approved</t>
+          <t>FIPS 140-3 path confirmed - BF-3 crypto module already approved</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3155,7 @@
       </c>
       <c r="B45" s="112" t="inlineStr">
         <is>
-          <t>If the primary gate is missed → stop before the $4.3M GA spend</t>
+          <t>If the primary gate is missed -&gt; stop before the $4.3M GA spend</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3201,7 @@
     <row r="1" ht="30" customHeight="1" s="79">
       <c r="A1" s="71" t="inlineStr">
         <is>
-          <t>Investment — dynamic cost model with drill-down</t>
+          <t>Investment - dynamic cost model with drill-down</t>
         </is>
       </c>
       <c r="B1" s="72" t="n"/>
@@ -3206,7 +3220,7 @@
     <row r="3" ht="20.1" customHeight="1" s="79">
       <c r="A3" s="81" t="inlineStr">
         <is>
-          <t>Cost summary  ·  rolls up from the drill-down blocks below</t>
+          <t>Cost summary - rolls up from the drill-down blocks below</t>
         </is>
       </c>
       <c r="B3" s="82" t="n"/>
@@ -3246,7 +3260,7 @@
     <row r="5" ht="15" customHeight="1" s="79">
       <c r="A5" s="86" t="inlineStr">
         <is>
-          <t>R&amp;D (engineers × role rate × years)</t>
+          <t>R&amp;D (engineers x role rate x years)</t>
         </is>
       </c>
       <c r="B5" s="23">
@@ -3272,7 +3286,7 @@
     <row r="6" ht="15" customHeight="1" s="79">
       <c r="A6" s="86" t="inlineStr">
         <is>
-          <t>Hardware engineering · thermal · FIPS</t>
+          <t>Hardware engineering - thermal - FIPS</t>
         </is>
       </c>
       <c r="B6" s="23">
@@ -3373,7 +3387,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Card bring-up · thermal · FIPS lab</t>
+          <t>Card bring-up - thermal - FIPS lab</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -3392,7 +3406,7 @@
     <row r="11" ht="20.1" customHeight="1" s="79">
       <c r="A11" s="83" t="inlineStr">
         <is>
-          <t>Drill-down A · R&amp;D engineer cost build-up</t>
+          <t>Drill-down A - R&amp;D engineer cost build-up</t>
         </is>
       </c>
       <c r="B11" s="74" t="n"/>
@@ -3466,7 +3480,7 @@
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>× of salary</t>
+          <t>x of salary</t>
         </is>
       </c>
       <c r="D14" s="24" t="n"/>
@@ -3589,7 +3603,7 @@
     <row r="19" ht="25.5" customHeight="1" s="79">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Duration (years)  =  months ÷ 12</t>
+          <t>Duration (years) = months / 12</t>
         </is>
       </c>
       <c r="B19" s="3">
@@ -3609,7 +3623,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Forward factor used by the role table: cost = engineers × rate/yr × years</t>
+          <t>Forward factor used by the role table: cost = engineers x rate/yr x years</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3659,7 @@
     <row r="21" ht="20.1" customHeight="1" s="79">
       <c r="A21" s="86" t="inlineStr">
         <is>
-          <t>Drill-down B · R&amp;D headcount by role (engineers should sum to the FTE above)</t>
+          <t>Drill-down B - R&amp;D headcount by role (engineers should sum to the FTE above)</t>
         </is>
       </c>
       <c r="B21" s="74" t="n"/>
@@ -3667,7 +3681,7 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>Loaded $/yr · per person</t>
+          <t>Loaded $/yr - per person</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
@@ -3709,7 +3723,7 @@
       </c>
       <c r="F23" s="24" t="inlineStr">
         <is>
-          <t>Driver/kernel specialists — rate above blended</t>
+          <t>Driver/kernel specialists - rate above blended</t>
         </is>
       </c>
     </row>
@@ -3736,7 +3750,7 @@
       </c>
       <c r="F24" s="24" t="inlineStr">
         <is>
-          <t>Senior core engineers — where most of the risk sits</t>
+          <t>Senior core engineers - where most of the risk sits</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3777,7 @@
       </c>
       <c r="F25" s="24" t="inlineStr">
         <is>
-          <t>RXP / compiler specialists — blended rate</t>
+          <t>RXP / compiler specialists - blended rate</t>
         </is>
       </c>
     </row>
@@ -3790,14 +3804,14 @@
       </c>
       <c r="F26" s="24" t="inlineStr">
         <is>
-          <t>QA / performance mix — below blended</t>
+          <t>QA / performance mix - below blended</t>
         </is>
       </c>
     </row>
     <row r="27" ht="25.5" customHeight="1" s="79">
       <c r="A27" s="86" t="inlineStr">
         <is>
-          <t>Subtotal R&amp;D  ·  flows to the Cost summary (R&amp;D row)</t>
+          <t>Subtotal R&amp;D - flows to the Cost summary (R&amp;D row)</t>
         </is>
       </c>
       <c r="B27" s="29">
@@ -3812,10 +3826,11 @@
       <c r="E27" s="24" t="n"/>
       <c r="F27" s="24" t="n"/>
     </row>
+    <row r="28"/>
     <row r="29" ht="20.1" customHeight="1" s="79">
       <c r="A29" s="85" t="inlineStr">
         <is>
-          <t>Drill-down C · Hardware engineering</t>
+          <t>Drill-down C - Hardware engineering</t>
         </is>
       </c>
       <c r="B29" s="82" t="n"/>
@@ -3951,15 +3966,16 @@
       </c>
       <c r="E34" s="30" t="inlineStr">
         <is>
-          <t>→ feeds the Cost summary</t>
+          <t>-&gt; feeds the Cost summary</t>
         </is>
       </c>
       <c r="F34" s="24" t="n"/>
     </row>
+    <row r="35"/>
     <row r="36" ht="20.1" customHeight="1" s="79">
       <c r="A36" s="85" t="inlineStr">
         <is>
-          <t>Drill-down D · Dev kits / NRE</t>
+          <t>Drill-down D - Dev kits / NRE</t>
         </is>
       </c>
       <c r="B36" s="82" t="n"/>
@@ -4122,15 +4138,16 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>→ feeds the Cost summary</t>
+          <t>-&gt; feeds the Cost summary</t>
         </is>
       </c>
       <c r="F42" s="24" t="n"/>
     </row>
+    <row r="43"/>
     <row r="44" ht="20.1" customHeight="1" s="79">
       <c r="A44" s="85" t="inlineStr">
         <is>
-          <t>Drill-down E · GTM / launch</t>
+          <t>Drill-down E - GTM / launch</t>
         </is>
       </c>
       <c r="B44" s="82" t="n"/>
@@ -4266,29 +4283,32 @@
       </c>
       <c r="E49" s="30" t="inlineStr">
         <is>
-          <t>→ feeds the Cost summary</t>
+          <t>-&gt; feeds the Cost summary</t>
         </is>
       </c>
       <c r="F49" s="24" t="n"/>
     </row>
+    <row r="50"/>
     <row r="51" ht="27.95" customHeight="1" s="79">
       <c r="A51" s="84" t="inlineStr">
         <is>
-          <t>How to play with it: change any cream cell (Base salary, Overhead, Engineers, a per-role $/yr rate, a Qty or a Unit cost) — the grey Cost/Amount/% cells, the subtotals and the grand Total all recalculate, and the Summary sheet follows.</t>
-        </is>
-      </c>
-    </row>
+          <t>How to play with it: change any cream cell (Base salary, Overhead, Engineers, a per-role $/yr rate, a Qty or a Unit cost) - the grey Cost/Amount/% cells, the subtotals and the grand Total all recalculate, and the Summary sheet follows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="87" t="inlineStr">
         <is>
-          <t>Check Point Software Technologies · Confidential   |   Barak Rozenfeld · Senior PM Assignment 2026   |   Slide 15   |   Cream = editable input · grey = formula (recalculates).</t>
-        </is>
-      </c>
-    </row>
+          <t>Check Point Software Technologies - Confidential | Barak Rozenfeld - Senior PM Assignment 2026 | Slide 15 | Cream = editable input - grey = formula (recalculates).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="97" t="inlineStr">
         <is>
-          <t>Phase split — what the $2.9M PoC covers vs the $4.3M to GA</t>
+          <t>Phase split - what the $2.9M PoC covers vs the $4.3M to GA</t>
         </is>
       </c>
       <c r="B55" s="98" t="n"/>
@@ -4300,7 +4320,7 @@
     <row r="56" ht="28" customHeight="1" s="79">
       <c r="A56" s="99" t="inlineStr">
         <is>
-          <t>PoC = first ~6 months · success gate 25 Gbps+ under TLS · if the gate is missed, we stop before the $4.3M GA spend. The split is a phase allocation of the same $7.2M program above.</t>
+          <t>PoC = first ~6 months - success gate 25 Gbps+ under TLS - if the gate is missed, we stop before the $4.3M GA spend. The split is a phase allocation of the same $7.2M program above.</t>
         </is>
       </c>
     </row>
@@ -4317,12 +4337,12 @@
       </c>
       <c r="C57" s="100" t="inlineStr">
         <is>
-          <t>PoC phase (≤6 mo)</t>
+          <t>PoC phase (&lt;=6 mo)</t>
         </is>
       </c>
       <c r="D57" s="100" t="inlineStr">
         <is>
-          <t>GA phase (≤12 mo)</t>
+          <t>GA phase (&lt;=12 mo)</t>
         </is>
       </c>
       <c r="E57" s="100" t="inlineStr">
@@ -4334,7 +4354,7 @@
     <row r="58">
       <c r="A58" s="101" t="inlineStr">
         <is>
-          <t>R&amp;D (engineers × rate × time)</t>
+          <t>R&amp;D (engineers x rate x time)</t>
         </is>
       </c>
       <c r="B58" s="102">
@@ -4351,14 +4371,14 @@
       </c>
       <c r="E58" s="99" t="inlineStr">
         <is>
-          <t>PoC runs a subset of the team — 10 eng × 6 mo (see build-up below)</t>
+          <t>PoC runs a subset of the team - 10 eng x 6 mo (see build-up below)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="101" t="inlineStr">
         <is>
-          <t>Hardware eng · thermal · FIPS</t>
+          <t>Hardware eng - thermal - FIPS</t>
         </is>
       </c>
       <c r="B59" s="102">
@@ -4444,14 +4464,15 @@
       </c>
       <c r="E62" s="106" t="inlineStr">
         <is>
-          <t>PoC ≈ $2.9M  ·  GA ≈ $4.3M  ·  total $7.2M</t>
-        </is>
-      </c>
-    </row>
+          <t>PoC ~ $2.9M - GA ~ $4.3M - total $7.2M</t>
+        </is>
+      </c>
+    </row>
+    <row r="63"/>
     <row r="64">
       <c r="A64" s="97" t="inlineStr">
         <is>
-          <t>PoC R&amp;D build-up  ·  drives the R&amp;D PoC cell above</t>
+          <t>PoC R&amp;D build-up - drives the R&amp;D PoC cell above</t>
         </is>
       </c>
       <c r="B64" s="98" t="n"/>
@@ -4499,7 +4520,7 @@
       </c>
       <c r="E66" s="99" t="inlineStr">
         <is>
-          <t>Focused subset — core offload + driver + perf</t>
+          <t>Focused subset - core offload + driver + perf</t>
         </is>
       </c>
     </row>
@@ -4546,7 +4567,7 @@
     <row r="69">
       <c r="A69" s="104" t="inlineStr">
         <is>
-          <t>PoC R&amp;D  =  engineers × months × rate</t>
+          <t>PoC R&amp;D = engineers x months x rate</t>
         </is>
       </c>
       <c r="B69" s="102">
@@ -4560,7 +4581,7 @@
       </c>
       <c r="E69" s="106" t="inlineStr">
         <is>
-          <t>≈ $1.25M — flows up to the R&amp;D PoC cell</t>
+          <t>~ $1.25M - flows up to the R&amp;D PoC cell</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4647,7 @@
     <row r="1" ht="30" customHeight="1" s="79">
       <c r="A1" s="71" t="inlineStr">
         <is>
-          <t>Delivery timeline — 18-month effort (with PoC gate)</t>
+          <t>Delivery timeline - 18-month effort (with PoC gate)</t>
         </is>
       </c>
       <c r="B1" s="72" t="n"/>
@@ -4644,6 +4665,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="27.95" customHeight="1" s="79">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -4702,7 +4724,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>M0 – M3</t>
+          <t>M0 - M3</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -4742,7 +4764,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>M3 – M8</t>
+          <t>M3 - M8</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -4769,7 +4791,7 @@
     <row r="7" ht="28.5" customHeight="1" s="79">
       <c r="A7" s="83" t="inlineStr">
         <is>
-          <t>Proof of Concept · TLS gate</t>
+          <t>Proof of Concept - TLS gate</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -4782,7 +4804,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>M8 – M10</t>
+          <t>M8 - M10</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -4814,7 +4836,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>IPS DB → RXP signature compiler; FIPS 140-3 filed early</t>
+          <t>IPS DB -&gt; RXP signature compiler; FIPS 140-3 filed early</t>
         </is>
       </c>
       <c r="C8" s="31" t="n">
@@ -4822,7 +4844,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>M10 – M14</t>
+          <t>M10 - M14</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -4849,7 +4871,7 @@
     <row r="9" ht="15" customHeight="1" s="79">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Beta → GA</t>
+          <t>Beta -&gt; GA</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
@@ -4862,7 +4884,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>M14 – M18</t>
+          <t>M14 - M18</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
@@ -4906,28 +4928,28 @@
     <row r="11" ht="15" customHeight="1" s="79">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>Note: effort months sum to 18; calendar windows overlap. FIPS 140-3 is submitted ≈ 9 months before GA (not after).</t>
+          <t>Note: effort months sum to 18; calendar windows overlap. FIPS 140-3 is submitted ~ 9 months before GA (not after).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" s="79">
       <c r="A12" s="84" t="inlineStr">
         <is>
-          <t>Note: effort months sum to 18; calendar windows overlap. The PoC (M8–M10) is a Go/No-Go gate — the project only commits to RXP/FIPS spend after 25G+ under TLS is demonstrated. FIPS 140-3 is submitted ≈ 9 months before GA.</t>
+          <t>Note: effort months sum to 18; calendar windows overlap. The PoC (M8-M10) is a Go/No-Go gate - the project only commits to RXP/FIPS spend after 25G+ under TLS is demonstrated. FIPS 140-3 is submitted ~ 9 months before GA.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="91" t="inlineStr">
         <is>
-          <t>Check Point Software Technologies · Confidential   |   Barak Rozenfeld · Senior PM Assignment 2026   |   Session 1 · Slide 15 — What it takes to deliver the solution   |   Edit the yellow input cells; grey cells are formulas.</t>
+          <t>Check Point Software Technologies - Confidential | Barak Rozenfeld - Senior PM Assignment 2026 | Session 1 - Slide 15 - What it takes to deliver the solution | Edit the yellow input cells; grey cells are formulas.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="87" t="inlineStr">
         <is>
-          <t>Check Point Software Technologies · Confidential   |   Barak Rozenfeld · Senior PM Assignment 2026   |   Slide 15   |   Cream = editable input · grey = formula (recalculates).</t>
+          <t>Check Point Software Technologies - Confidential | Barak Rozenfeld - Senior PM Assignment 2026 | Slide 15 | Cream = editable input - grey = formula (recalculates).</t>
         </is>
       </c>
     </row>
@@ -4980,10 +5002,11 @@
     <row r="2" ht="18" customHeight="1" s="79">
       <c r="A2" s="78" t="inlineStr">
         <is>
-          <t>Hardware, software/integration and product readiness — each with a target metric, its basis/source and the assumption to validate.</t>
-        </is>
-      </c>
-    </row>
+          <t>Hardware, software/integration and product readiness - each with a target metric, its basis/source and the assumption to validate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="79">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -5062,7 +5085,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>≤ ~75W added</t>
+          <t>&lt;= ~75W added</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -5072,7 +5095,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Early thermal sim; if no headroom → factory option next gen</t>
+          <t>Early thermal sim; if no headroom -&gt; factory option next gen</t>
         </is>
       </c>
     </row>
@@ -5145,12 +5168,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>The API between CoreXL and the card — most of the 12 engineers</t>
+          <t>The API between CoreXL and the card - most of the 12 engineers</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>TP ≥ 25G under TLS</t>
+          <t>TP &gt;= 25G under TLS</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -5173,7 +5196,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Converting the IPS DB → RXP; metric is % of signatures that compile</t>
+          <t>Converting the IPS DB -&gt; RXP; metric is % of signatures that compile</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -5188,7 +5211,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Partial IPS acceptable — TLS offload delivers most of the gain</t>
+          <t>Partial IPS acceptable - TLS offload delivers most of the gain</t>
         </is>
       </c>
     </row>
@@ -5205,7 +5228,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Maintain FIPS 140-3; assess the card’s impact on CC certification</t>
+          <t>Maintain FIPS 140-3; assess the card's impact on CC certification</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -5266,7 +5289,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Beta → GA</t>
+          <t>Beta -&gt; GA</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -5280,10 +5303,11 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="91" t="inlineStr">
         <is>
-          <t>Check Point Software Technologies · Confidential   |   Barak Rozenfeld · Senior PM Assignment 2026   |   Session 1 · Slide 15 — What it takes to deliver the solution   |   Edit the yellow input cells; grey cells are formulas.</t>
+          <t>Check Point Software Technologies - Confidential | Barak Rozenfeld - Senior PM Assignment 2026 | Session 1 - Slide 15 - What it takes to deliver the solution | Edit the yellow input cells; grey cells are formulas.</t>
         </is>
       </c>
       <c r="B15" s="74" t="n"/>
@@ -5354,10 +5378,11 @@
     <row r="2" ht="17.1" customHeight="1" s="79">
       <c r="A2" s="78" t="inlineStr">
         <is>
-          <t>Severity × Likelihood (High=3, Medium=2, Low=1; Score = S×L). Each risk carries its basis/source, mitigation and a measurable target.</t>
-        </is>
-      </c>
-    </row>
+          <t>Severity x Likelihood (High=3, Medium=2, Low=1; Score = SxL). Each risk carries its basis/source, mitigation and a measurable target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="27.95" customHeight="1" s="79">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -5469,7 +5494,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Only part of the IPS signatures compile to RXP → partial IPS gain</t>
+          <t>Only part of the IPS signatures compile to RXP -&gt; partial IPS gain</t>
         </is>
       </c>
       <c r="D6" s="35" t="inlineStr">
@@ -5535,7 +5560,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Early thermal simulation; if no headroom → factory option next generation</t>
+          <t>Early thermal simulation; if no headroom -&gt; factory option next generation</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -5650,17 +5675,19 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="92" t="inlineStr">
         <is>
-          <t>Legend — Severity/Likelihood: High (3) · Medium (2) · Low (1). Score 6 = red, 3–4 = amber, 1–2 = green. Risk severity ranking is a qualitative assessment.</t>
-        </is>
-      </c>
-    </row>
+          <t>Legend - Severity/Likelihood: High (3) - Medium (2) - Low (1). Score 6 = red, 3-4 = amber, 1-2 = green. Risk severity ranking is a qualitative assessment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="91" t="inlineStr">
         <is>
-          <t>Check Point Software Technologies · Confidential   |   Barak Rozenfeld · Senior PM Assignment 2026   |   Slide 15   |   Cream = editable input · grey = formula (recalculates).</t>
+          <t>Check Point Software Technologies - Confidential | Barak Rozenfeld - Senior PM Assignment 2026 | Slide 15 | Cream = editable input - grey = formula (recalculates).</t>
         </is>
       </c>
       <c r="B13" s="74" t="n"/>
@@ -5711,7 +5738,7 @@
     <row r="1" ht="30" customHeight="1" s="79">
       <c r="A1" s="93" t="inlineStr">
         <is>
-          <t>ROI — 3-year business case (expanded from Slide 16)</t>
+          <t>ROI - 3-year business case (expanded from Slide 16)</t>
         </is>
       </c>
       <c r="B1" s="72" t="n"/>
@@ -5723,14 +5750,15 @@
     <row r="2" ht="27.95" customHeight="1" s="79">
       <c r="A2" s="80" t="inlineStr">
         <is>
-          <t>Why the numbers, how they are built, and the sales assumptions (incl. 29100/29200 cannibalization). Cream = editable input · grey = formula. The one-time investment links live to the Investment sheet.</t>
-        </is>
-      </c>
-    </row>
+          <t>Why the numbers, how they are built, and the sales assumptions (incl. 29100/29200 cannibalization). Cream = editable input - grey = formula. The one-time investment links live to the Investment sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="21.95" customHeight="1" s="79">
       <c r="A4" s="77" t="inlineStr">
         <is>
-          <t>Headline — 3-year outcome (base vs. base + deal upside)</t>
+          <t>Headline - 3-year outcome (base vs. base + deal upside)</t>
         </is>
       </c>
       <c r="B4" s="74" t="n"/>
@@ -5862,12 +5890,12 @@
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>Net ÷ investment</t>
+          <t>Net / investment</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Net ÷ investment, net of cannibalization; deck shows ~189% / ~408% (sheet exact)</t>
+          <t>Net / investment, net of cannibalization; deck shows ~189% / ~408% (sheet exact)</t>
         </is>
       </c>
     </row>
@@ -5882,7 +5910,7 @@
       </c>
       <c r="C10" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D10" s="4" t="n"/>
@@ -5897,10 +5925,11 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="21.95" customHeight="1" s="79">
       <c r="A12" s="77" t="inlineStr">
         <is>
-          <t>Key inputs — editable (cream); each with its basis and assumption</t>
+          <t>Key inputs - editable (cream); each with its basis and assumption</t>
         </is>
       </c>
       <c r="B12" s="74" t="n"/>
@@ -5992,7 +6021,7 @@
     <row r="16" ht="24" customHeight="1" s="79">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Attach rate — year 1</t>
+          <t>Attach rate - year 1</t>
         </is>
       </c>
       <c r="B16" s="47" t="n">
@@ -6018,7 +6047,7 @@
     <row r="17" ht="24" customHeight="1" s="79">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Attach rate — year 2</t>
+          <t>Attach rate - year 2</t>
         </is>
       </c>
       <c r="B17" s="47" t="n">
@@ -6044,7 +6073,7 @@
     <row r="18" ht="24" customHeight="1" s="79">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Attach rate — year 3</t>
+          <t>Attach rate - year 3</t>
         </is>
       </c>
       <c r="B18" s="47" t="n">
@@ -6096,7 +6125,7 @@
     <row r="20" ht="24" customHeight="1" s="79">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Gross margin — module</t>
+          <t>Gross margin - module</t>
         </is>
       </c>
       <c r="B20" s="47" t="n">
@@ -6122,7 +6151,7 @@
     <row r="21" ht="24" customHeight="1" s="79">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Gross margin — DC/HQ deal</t>
+          <t>Gross margin - DC/HQ deal</t>
         </is>
       </c>
       <c r="B21" s="47" t="n">
@@ -6152,7 +6181,7 @@
         </is>
       </c>
       <c r="B22" s="40">
-        <f>'2 · Investment'!B9</f>
+        <f>'2. Investment'!B9</f>
         <v/>
       </c>
       <c r="C22" s="45" t="inlineStr">
@@ -6163,7 +6192,7 @@
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>Live link → '2 · Investment'!B9</t>
+          <t>Live link -&gt; '2 - Investment'!B9</t>
         </is>
       </c>
       <c r="F22" s="18" t="inlineStr">
@@ -6220,7 +6249,7 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>Incremental wins from the 4× TP+TLS advantage</t>
+          <t>Incremental wins from the 4x TP+TLS advantage</t>
         </is>
       </c>
     </row>
@@ -6250,10 +6279,11 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="21.95" customHeight="1" s="79">
       <c r="A27" s="77" t="inlineStr">
         <is>
-          <t>Build-up A — attach on new units (how 1,800 modules &amp; $27.0M arise)</t>
+          <t>Build-up A - attach on new units (how 1,800 modules &amp; $27.0M arise)</t>
         </is>
       </c>
       <c r="B27" s="74" t="n"/>
@@ -6396,14 +6426,15 @@
       </c>
       <c r="F32" s="18" t="inlineStr">
         <is>
-          <t>1,800 modules over 3 years as attach grows 30% → 50%</t>
-        </is>
-      </c>
-    </row>
+          <t>1,800 modules over 3 years as attach grows 30% -&gt; 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
     <row r="34" ht="21.95" customHeight="1" s="79">
       <c r="A34" s="77" t="inlineStr">
         <is>
-          <t>Build-up B — base module revenue (3 years)</t>
+          <t>Build-up B - base module revenue (3 years)</t>
         </is>
       </c>
       <c r="B34" s="74" t="n"/>
@@ -6462,7 +6493,7 @@
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>New-unit attach, years 1–3</t>
+          <t>New-unit attach, years 1-3</t>
         </is>
       </c>
     </row>
@@ -6488,7 +6519,7 @@
       </c>
       <c r="F37" s="18" t="inlineStr">
         <is>
-          <t>925 upgrades × $15K; demand concentrated in year 1</t>
+          <t>925 upgrades x $15K; demand concentrated in year 1</t>
         </is>
       </c>
     </row>
@@ -6514,10 +6545,11 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40" ht="21.95" customHeight="1" s="79">
       <c r="A40" s="77" t="inlineStr">
         <is>
-          <t>ROI waterfall — base vs. base + deal upside</t>
+          <t>ROI waterfall - base vs. base + deal upside</t>
         </is>
       </c>
       <c r="B40" s="74" t="n"/>
@@ -6601,7 +6633,7 @@
       </c>
       <c r="F43" s="18" t="inlineStr">
         <is>
-          <t>75 deals (25/yr × 3) × $350K</t>
+          <t>75 deals (25/yr x 3) x $350K</t>
         </is>
       </c>
     </row>
@@ -6649,7 +6681,7 @@
       </c>
       <c r="F45" s="18" t="inlineStr">
         <is>
-          <t>65% module · 60% deal</t>
+          <t>65% module - 60% deal</t>
         </is>
       </c>
     </row>
@@ -6718,7 +6750,7 @@
       <c r="D48" s="4" t="n"/>
       <c r="E48" s="19" t="inlineStr">
         <is>
-          <t>Net ÷ investment</t>
+          <t>Net / investment</t>
         </is>
       </c>
       <c r="F48" s="18" t="inlineStr">
@@ -6738,7 +6770,7 @@
       </c>
       <c r="C49" s="43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D49" s="4" t="n"/>
@@ -6753,10 +6785,11 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51" ht="21.95" customHeight="1" s="79">
       <c r="A51" s="77" t="inlineStr">
         <is>
-          <t>Sales adjustment — 29100/29200 cannibalization (now netted into the headline ROI)</t>
+          <t>Sales adjustment - 29100/29200 cannibalization (now netted into the headline ROI)</t>
         </is>
       </c>
       <c r="B51" s="74" t="n"/>
@@ -6848,7 +6881,7 @@
       </c>
       <c r="F55" s="18" t="inlineStr">
         <is>
-          <t>Enterprise appliance; varies by bundle/region/discount — placeholder to edit</t>
+          <t>Enterprise appliance; varies by bundle/region/discount - placeholder to edit</t>
         </is>
       </c>
     </row>
@@ -6973,7 +7006,7 @@
     <row r="61" ht="21.95" customHeight="1" s="79">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Memo · net contribution before cannibalization (gross)</t>
+          <t>Memo - net contribution before cannibalization (gross)</t>
         </is>
       </c>
       <c r="B61" s="40">
@@ -6996,7 +7029,7 @@
     <row r="62" ht="24" customHeight="1" s="79">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Memo · ROI before cannibalization (gross)</t>
+          <t>Memo - ROI before cannibalization (gross)</t>
         </is>
       </c>
       <c r="B62" s="41">
@@ -7007,7 +7040,7 @@
       <c r="D62" s="4" t="n"/>
       <c r="E62" s="19" t="inlineStr">
         <is>
-          <t>Adjusted net ÷ investment</t>
+          <t>Adjusted net / investment</t>
         </is>
       </c>
       <c r="F62" s="18" t="inlineStr">
@@ -7016,10 +7049,11 @@
         </is>
       </c>
     </row>
+    <row r="63"/>
     <row r="64" ht="21.95" customHeight="1" s="79">
       <c r="A64" s="80" t="inlineStr">
         <is>
-          <t>Check Point Software Technologies · Confidential   |   Barak Rozenfeld · Senior PM Assignment 2026   |   Slide 16   |   Cream = editable input · grey = formula (recalculates).</t>
+          <t>Check Point Software Technologies - Confidential | Barak Rozenfeld - Senior PM Assignment 2026 | Slide 16 | Cream = editable input - grey = formula (recalculates).</t>
         </is>
       </c>
     </row>
@@ -7061,7 +7095,7 @@
     <row r="1" ht="16.5" customHeight="1" s="79">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>Slide 12 — Four alternatives for accelerating TP under TLS</t>
+          <t>Slide 12 - Four alternatives for accelerating TP under TLS</t>
         </is>
       </c>
     </row>
@@ -7072,6 +7106,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
         <is>
@@ -7100,7 +7135,7 @@
       </c>
       <c r="F4" s="63" t="inlineStr">
         <is>
-          <t>Throughput (today 10)  &amp;  verdict</t>
+          <t>Throughput (today 10) &amp; verdict</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7157,7 @@
       </c>
       <c r="D5" s="96" t="inlineStr">
         <is>
-          <t>3–5 years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="E5" s="96" t="inlineStr">
@@ -7132,7 +7167,7 @@
       </c>
       <c r="F5" s="65" t="inlineStr">
         <is>
-          <t>~40+ · Rejected — cost &amp; time prohibitive, inflexible</t>
+          <t>~40+ - Rejected - cost &amp; time prohibitive, inflexible</t>
         </is>
       </c>
     </row>
@@ -7159,12 +7194,12 @@
       </c>
       <c r="E6" s="96" t="inlineStr">
         <is>
-          <t>$30–50M</t>
+          <t>$30-50M</t>
         </is>
       </c>
       <c r="F6" s="65" t="inlineStr">
         <is>
-          <t>~30–40 · Rejected — costly, HDL per engine</t>
+          <t>~30-40 - Rejected - costly, HDL per engine</t>
         </is>
       </c>
     </row>
@@ -7196,7 +7231,7 @@
       </c>
       <c r="F7" s="65" t="inlineStr">
         <is>
-          <t>10→~20 (×2) · Rejected — crypto only, no Arm cores</t>
+          <t>10-&gt;~20 (x2) - Rejected - crypto only, no Arm cores</t>
         </is>
       </c>
     </row>
@@ -7228,10 +7263,11 @@
       </c>
       <c r="F8" s="67" t="inlineStr">
         <is>
-          <t>10→~40 (×4) · CHOSEN — best TP/RU + software-updatable</t>
-        </is>
-      </c>
-    </row>
+          <t>10-&gt;~40 (x4) - CHOSEN - best TP/RU + software-updatable</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="95" t="inlineStr">
         <is>
@@ -7266,17 +7302,18 @@
     <row r="1" ht="16.5" customHeight="1" s="79">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>Alternative 1 — Build our own ASIC</t>
+          <t>Alternative 1 - Build our own ASIC</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" s="79">
       <c r="A2" s="94" t="inlineStr">
         <is>
-          <t>A Check Point-designed dedicated chip. Rejected: cost and time are prohibitive and the logic is burned into silicon — a new engine means a whole new hardware generation.</t>
-        </is>
-      </c>
-    </row>
+          <t>A Check Point-designed dedicated chip. Rejected: cost and time are prohibitive and the logic is burned into silicon - a new engine means a whole new hardware generation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="55" t="inlineStr">
         <is>
@@ -7314,7 +7351,7 @@
       </c>
       <c r="B6" s="59" t="inlineStr">
         <is>
-          <t>3–5 years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="C6" s="96" t="inlineStr">
@@ -7374,6 +7411,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="55" t="inlineStr">
         <is>
@@ -7445,7 +7483,7 @@
       </c>
       <c r="B15" s="58" t="inlineStr">
         <is>
-          <t>~6–12 months</t>
+          <t>~6-12 months</t>
         </is>
       </c>
       <c r="C15" s="95" t="inlineStr">
@@ -7479,7 +7517,7 @@
       </c>
       <c r="B17" s="58" t="inlineStr">
         <is>
-          <t>~6–12 months</t>
+          <t>~6-12 months</t>
         </is>
       </c>
       <c r="C17" s="95" t="inlineStr">
@@ -7496,7 +7534,7 @@
       </c>
       <c r="B18" s="58" t="inlineStr">
         <is>
-          <t>~6–12 months</t>
+          <t>~6-12 months</t>
         </is>
       </c>
       <c r="C18" s="95" t="inlineStr">
@@ -7513,7 +7551,7 @@
       </c>
       <c r="B19" s="58" t="inlineStr">
         <is>
-          <t>3–5 years</t>
+          <t>3-5 years</t>
         </is>
       </c>
       <c r="C19" s="95" t="inlineStr">
@@ -7522,6 +7560,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="55" t="inlineStr">
         <is>
@@ -7592,7 +7631,7 @@
       </c>
       <c r="C25" s="95" t="inlineStr">
         <is>
-          <t>Masks alone ~$15–25M at 7nm, plus place-and-route</t>
+          <t>Masks alone ~$15-25M at 7nm, plus place-and-route</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7646,7 @@
       </c>
       <c r="C26" s="95" t="inlineStr">
         <is>
-          <t>Each respin ~$5–15M in masks + lost time</t>
+          <t>Each respin ~$5-15M in masks + lost time</t>
         </is>
       </c>
     </row>
@@ -7644,7 +7683,7 @@
     <row r="29">
       <c r="A29" s="58" t="inlineStr">
         <is>
-          <t>Total NRE  (≈ IBS/McKinsey 7nm)</t>
+          <t>Total NRE (~ IBS/McKinsey 7nm)</t>
         </is>
       </c>
       <c r="B29" s="69">
@@ -7701,17 +7740,18 @@
     <row r="1" ht="16.5" customHeight="1" s="79">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>Alternative 2 — Self-designed FPGA</t>
+          <t>Alternative 2 - Self-designed FPGA</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" s="79">
       <c r="A2" s="94" t="inlineStr">
         <is>
-          <t>An FPGA designed by Check Point. Rejected: still costly, every new engine needs fresh HDL work, and performance trails a custom ASIC. The $30–50M range below is built bottom-up to a ~$40M midpoint.</t>
-        </is>
-      </c>
-    </row>
+          <t>An FPGA designed by Check Point. Rejected: still costly, every new engine needs fresh HDL work, and performance trails a custom ASIC. The $30-50M range below is built bottom-up to a ~$40M midpoint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="55" t="inlineStr">
         <is>
@@ -7766,7 +7806,7 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>$30–50M</t>
+          <t>$30-50M</t>
         </is>
       </c>
       <c r="C7" s="96" t="inlineStr">
@@ -7783,7 +7823,7 @@
       </c>
       <c r="B8" s="59" t="inlineStr">
         <is>
-          <t>~30–40</t>
+          <t>~30-40</t>
         </is>
       </c>
       <c r="C8" s="96" t="inlineStr">
@@ -7809,6 +7849,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="55" t="inlineStr">
         <is>
@@ -7846,7 +7887,7 @@
       </c>
       <c r="B13" s="58" t="inlineStr">
         <is>
-          <t>~12–15 months</t>
+          <t>~12-15 months</t>
         </is>
       </c>
       <c r="C13" s="95" t="inlineStr">
@@ -7863,7 +7904,7 @@
       </c>
       <c r="B14" s="58" t="inlineStr">
         <is>
-          <t>~9–12 months</t>
+          <t>~9-12 months</t>
         </is>
       </c>
       <c r="C14" s="95" t="inlineStr">
@@ -7880,7 +7921,7 @@
       </c>
       <c r="B15" s="58" t="inlineStr">
         <is>
-          <t>~6–9 months</t>
+          <t>~6-9 months</t>
         </is>
       </c>
       <c r="C15" s="95" t="inlineStr">
@@ -7936,10 +7977,11 @@
       </c>
       <c r="C18" s="95" t="inlineStr">
         <is>
-          <t>No tape-out, so ~1–2 yr shorter than an ASIC</t>
-        </is>
-      </c>
-    </row>
+          <t>No tape-out, so ~1-2 yr shorter than an ASIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="55" t="inlineStr">
         <is>
@@ -7972,7 +8014,7 @@
     <row r="22">
       <c r="A22" s="61" t="inlineStr">
         <is>
-          <t>FTE — HDL/verif/firmware/board team</t>
+          <t>FTE - HDL/verif/firmware/board team</t>
         </is>
       </c>
       <c r="B22" s="70" t="n">
@@ -8052,7 +8094,7 @@
       </c>
       <c r="C27" s="95" t="inlineStr">
         <is>
-          <t>Main swing factor for the $30–50M range</t>
+          <t>Main swing factor for the $30-50M range</t>
         </is>
       </c>
     </row>
@@ -8104,7 +8146,7 @@
     <row r="31">
       <c r="A31" s="58" t="inlineStr">
         <is>
-          <t>Total NRE  (midpoint of $30–50M)</t>
+          <t>Total NRE (midpoint of $30-50M)</t>
         </is>
       </c>
       <c r="B31" s="69">
@@ -8113,7 +8155,7 @@
       </c>
       <c r="C31" s="95" t="inlineStr">
         <is>
-          <t>≈$40M; 20 FTE &amp; fewer respins → ~$30M, 30 FTE &amp; more → ~$50M</t>
+          <t>~$40M; 20 FTE &amp; fewer respins -&gt; ~$30M, 30 FTE &amp; more -&gt; ~$50M</t>
         </is>
       </c>
     </row>

</xml_diff>